<commit_message>
input and results after modification of PR function adn amin script
</commit_message>
<xml_diff>
--- a/input/input_PR_pure.xlsx
+++ b/input/input_PR_pure.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/02_UHS EXPERIMENTS/H2 DISPLACEMENT EXPERIMENT/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pennstateoffice365-my.sharepoint.com/personal/izg5132_psu_edu/Documents/06_PHD_EME_PSU/00 RESEARCH/PHD UHS PROJECT/MATLAB-GITHUB/UHS-CF-Dispersion-Exps/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE3ED494-FEE3-4BE4-A9E3-8A2DDC2A6C0D}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="11_F25DC773A252ABDACC10485949585E945ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{788167F7-1CF7-4EF9-A280-851C920EE6C2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -41,9 +41,6 @@
     <t>Fluid</t>
   </si>
   <si>
-    <t>Acentric factor</t>
-  </si>
-  <si>
     <t>H2</t>
   </si>
   <si>
@@ -78,6 +75,9 @@
   </si>
   <si>
     <t>kg/mol</t>
+  </si>
+  <si>
+    <t>Acentric Factor</t>
   </si>
 </sst>
 </file>
@@ -407,32 +407,32 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
       <c r="E1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3">
         <f>2.016*(10^-3)</f>
@@ -450,7 +450,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <f>44.01*(10^-3)</f>
@@ -468,7 +468,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <v>4.0000000000000001E-3</v>
@@ -485,7 +485,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6">
         <v>0.13128999999999999</v>
@@ -502,7 +502,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7">
         <v>1.6039999999999999E-2</v>
@@ -519,7 +519,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>2.8014000000000001E-2</v>

</xml_diff>